<commit_message>
test(v5): verify full C16 capture ownership and expose complete OOC DRC
</commit_message>
<xml_diff>
--- a/v5/hardware/bom/working/2026-10-10/BOM_AX7020_NU40C10T_AD7606C16_WORKING.xlsx
+++ b/v5/hardware/bom/working/2026-10-10/BOM_AX7020_NU40C10T_AD7606C16_WORKING.xlsx
@@ -2,13 +2,13 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="R8117df44e68b4481"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upper" sheetId="2" r:id="R80d1fc1f65b248db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lower" sheetId="3" r:id="Re45f8aba2b8949e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Central" sheetId="4" r:id="R190a24261e6749ce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External" sheetId="5" r:id="Rd95e09b2628c4fcf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_References" sheetId="6" r:id="R5262b605feba4a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="R183a8551ae2449d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="1" r:id="Rd899f0fda2f7484c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Upper" sheetId="2" r:id="Rd390cc81793840b4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lower" sheetId="3" r:id="Rbd98c7edcd574134"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Central" sheetId="4" r:id="R7aa1ba16c5d04338"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External" sheetId="5" r:id="R48fc42d9e2b44fe9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_References" sheetId="6" r:id="Rc22b943855684973"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="7" r:id="Rb685660880b94c45"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2470,7 +2470,7 @@
         <x:v>Alternative / required evidence</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="76" customHeight="1">
+    <x:row r="5" ht="192" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>B-001</x:v>
       </x:c>
@@ -2572,7 +2572,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="76" customHeight="1">
+    <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>B-003</x:v>
       </x:c>
@@ -3949,7 +3949,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="76" customHeight="1">
+    <x:row r="34" ht="204" customHeight="1">
       <x:c r="A34" s="7" t="str">
         <x:v>B-046</x:v>
       </x:c>
@@ -4000,7 +4000,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="76" customHeight="1">
+    <x:row r="35" ht="96" customHeight="1">
       <x:c r="A35" s="7" t="str">
         <x:v>B-047</x:v>
       </x:c>
@@ -4357,7 +4357,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="76" customHeight="1">
+    <x:row r="42" ht="252" customHeight="1">
       <x:c r="A42" s="7" t="str">
         <x:v>B-054</x:v>
       </x:c>
@@ -4714,7 +4714,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="76" customHeight="1">
+    <x:row r="49" ht="204" customHeight="1">
       <x:c r="A49" s="7" t="str">
         <x:v>B-061</x:v>
       </x:c>
@@ -6049,7 +6049,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0d9d70a20ccc49b8"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9af50fb3e63a4036"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6182,7 +6182,7 @@
         <x:v>Alternative / required evidence</x:v>
       </x:c>
     </x:row>
-    <x:row r="5" ht="76" customHeight="1">
+    <x:row r="5" ht="192" customHeight="1">
       <x:c r="A5" s="7" t="str">
         <x:v>B-001</x:v>
       </x:c>
@@ -6284,7 +6284,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="7" ht="76" customHeight="1">
+    <x:row r="7" ht="96" customHeight="1">
       <x:c r="A7" s="7" t="str">
         <x:v>B-003</x:v>
       </x:c>
@@ -7661,7 +7661,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="34" ht="76" customHeight="1">
+    <x:row r="34" ht="204" customHeight="1">
       <x:c r="A34" s="7" t="str">
         <x:v>B-046</x:v>
       </x:c>
@@ -7712,7 +7712,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="35" ht="76" customHeight="1">
+    <x:row r="35" ht="96" customHeight="1">
       <x:c r="A35" s="7" t="str">
         <x:v>B-047</x:v>
       </x:c>
@@ -8069,7 +8069,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="76" customHeight="1">
+    <x:row r="42" ht="252" customHeight="1">
       <x:c r="A42" s="7" t="str">
         <x:v>B-054</x:v>
       </x:c>
@@ -8426,7 +8426,7 @@
         <x:v>Inherited candidate quantity; netlist/thermal review pending</x:v>
       </x:c>
     </x:row>
-    <x:row r="49" ht="76" customHeight="1">
+    <x:row r="49" ht="204" customHeight="1">
       <x:c r="A49" s="7" t="str">
         <x:v>B-061</x:v>
       </x:c>
@@ -9761,7 +9761,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbfa280ce02644414"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R370162ef90ca43a9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -12648,7 +12648,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5ae3d4d80dbd4c9c"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9fc7fa8d17ef48ea"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -14776,7 +14776,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1b1d7fc0f16f4ed7"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rd2cb434f2de54375"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>